<commit_message>
Review-board (#31): make synthetic plate invalid-by-construction; reconcile real-make rule
- model.py _plate: switch to a 2-letter/4-digit/2-letter pattern, which is not a live registration
  format in any corpus country (DE/FR/ES/IT/NL/IE) — so it cannot match a real plate (the board noted
  the old AB-123-CD was exactly the live French SIV format). Same invalid-by-construction principle as
  the national IDs. (No RNG-stream change — same number of draws — so only plate strings differ.)
- CLAUDE.md: clarify the "no real persons/companies" hard rule so it's consistent with the corpus —
  it targets fabricated records/parties about real entities; incidental factual references (a vehicle
  make) are fine; the corpus should carry realistic synthetic PII (redaction is the RAG layer's job).
</commit_message>
<xml_diff>
--- a/sample/docs/tabular/loss-run.xlsx
+++ b/sample/docs/tabular/loss-run.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2023-10-10</t>
+          <t>2024-01-11</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>slip and fall</t>
+          <t>burglary</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -512,7 +512,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>8550</v>
+        <v>23700</v>
       </c>
     </row>
     <row r="4">
@@ -523,22 +523,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>COM-0000004</t>
+          <t>HH-0000001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Household</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2024-07-04</t>
+          <t>2024-06-21</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>burglary</t>
+          <t>theft</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -547,10 +547,10 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>53950</v>
+        <v>12850</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>19694.51</v>
+        <v>4474.47</v>
       </c>
     </row>
     <row r="5">

</xml_diff>